<commit_message>
Continuous heat-map chart, merged ID-by-Region tab, indeterminate fix
- Region Distribution: new continuous heat-map (version B) replaces the
  discrete-bucket chart (version A hidden). Scale runs 2 -> max share-count
  with a colour bar; segments >=10% labelled with % and code / "N codes".
- Merged the Single-region power chart into the same tab, renamed
  "Identification by Region".
- Pack inventory: M3/M6H/M10 reclassified from "makhfi unknown" to
  "indeterminate" in wolves_data.xlsx (indeterminate sentinel now 7).
- Regenerated data_table.html and the QC / verification / inference reports.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wolves_data.xlsx
+++ b/wolves_data.xlsx
@@ -1766,7 +1766,7 @@
       </c>
       <c r="I4" s="0" t="inlineStr">
         <is>
-          <t>makhfi unknown</t>
+          <t>indeterminate</t>
         </is>
       </c>
       <c r="K4" s="0" t="inlineStr">
@@ -2137,7 +2137,7 @@
       </c>
       <c r="I7" s="0" t="inlineStr">
         <is>
-          <t>makhfi unknown</t>
+          <t>indeterminate</t>
         </is>
       </c>
       <c r="L7" s="0" t="inlineStr">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="I11" s="0" t="inlineStr">
         <is>
-          <t>makhfi unknown</t>
+          <t>indeterminate</t>
         </is>
       </c>
       <c r="L11" s="0" t="inlineStr">

</xml_diff>